<commit_message>
2 agents completing the tasks
</commit_message>
<xml_diff>
--- a/src/main/resources/test_cases.xlsx
+++ b/src/main/resources/test_cases.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sysco-my.sharepoint.com/personal/cgov4385_sysco_com/Documents/Chiran/UI Action Adapter/Playwright UI Action Adapter/src/main/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="92" documentId="11_0DD0DCC95515360C39875808F5570708BA4E2934" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57AEDF9F-874D-41DE-87CD-0C65E4A3940A}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="11_0DD0DCC95515360C39875808F5570708BA4E2934" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE5FAA75-0219-4B1E-9738-E9AB42B4FDEB}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-25230" yWindow="1755" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="122">
   <si>
     <t>Issue Key</t>
   </si>
@@ -223,9 +224,6 @@
     <t>Authentication request is processed successfully without credential errors.</t>
   </si>
   <si>
-    <t>Authentication completes successfully and the user is redirected back to the application.</t>
-  </si>
-  <si>
     <t>The user successfully lands on the RPA Dashboard QA home page.</t>
   </si>
   <si>
@@ -250,18 +248,9 @@
     <t>User is redirected to Microsoft SSO authentication in a new popup window.</t>
   </si>
   <si>
-    <t>Username is accepted without validation errors.</t>
-  </si>
-  <si>
     <t>On the Microsoft SSO page which is a new popup page so you have to have navigate that tab, click the 'Yes' button.</t>
   </si>
   <si>
-    <t>there should be only one tab available now</t>
-  </si>
-  <si>
-    <t>Verify the user is redirected back to the RPA Dashboard QA environment. if you see any pop up alert on there click it on the 'OK' button .And if you see it is still login button visible click it.</t>
-  </si>
-  <si>
     <t>Click the 'Bots' text or Bots icon from the left-side navigation menu.</t>
   </si>
   <si>
@@ -274,21 +263,9 @@
     <t>Should navigate to sysco network id page.</t>
   </si>
   <si>
-    <t>wait for 5 second and click the login button</t>
-  </si>
-  <si>
-    <t>Should wait untill waits is happening</t>
-  </si>
-  <si>
-    <t>check the visibility os the home text if it not visible you need to click the login button again. Then click the home text on the left side and then click the  bots text</t>
-  </si>
-  <si>
     <t>Email: Chiran.Govinnage@sysco.com; Network ID: cgov4385 ; Bot: CECE ;  RPA Dashboard QA URL : https://dashboard-qa.000-rpa-np.centralus.azr.sysco.net/</t>
   </si>
   <si>
-    <t>check the avaialility of Microsoft SSO page screen if it is then close that TAB</t>
-  </si>
-  <si>
     <t>SE-TC-001</t>
   </si>
   <si>
@@ -397,7 +374,19 @@
     <t>On the Microsoft SSO page which is a new popup page so you have to have navigate that tab, Enter password.  just one input field will be available.and click the 'Sign in' button.</t>
   </si>
   <si>
-    <t>On the Microsoft SSO page which is a new popup page so you have to have navigate that tab, Enter 'cgov4385' wait there few moment. There will not be any place holders there.</t>
+    <t xml:space="preserve"> if you see any pop up alert on there click it on the 'OK' button .And if you see it is still login button visible click it.</t>
+  </si>
+  <si>
+    <t>Verify the user is redirected back to the RPA Dashboard QA environment.</t>
+  </si>
+  <si>
+    <t>click login button</t>
+  </si>
+  <si>
+    <t>home page should be visible</t>
+  </si>
+  <si>
+    <t>test ened</t>
   </si>
 </sst>
 </file>
@@ -786,7 +775,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:AS24"/>
+  <dimension ref="A1:AS21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" bestFit="1" customWidth="1"/>
@@ -969,7 +958,7 @@
         <v>54</v>
       </c>
       <c r="O2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="P2" t="s">
         <v>55</v>
@@ -1020,7 +1009,7 @@
         <v>50</v>
       </c>
       <c r="AF2" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="AG2" s="5" t="s">
         <v>65</v>
@@ -1046,221 +1035,109 @@
     </row>
     <row r="3" spans="1:45" ht="45" x14ac:dyDescent="0.25">
       <c r="AF3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="AG3" s="5" t="s">
         <v>72</v>
-      </c>
-      <c r="AG3" s="5" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:45" ht="30" x14ac:dyDescent="0.25">
       <c r="AF4" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="AG4" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="AG4" s="5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:45" ht="75" x14ac:dyDescent="0.25">
       <c r="AF5" s="5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="AG5" s="5" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:45" ht="45" x14ac:dyDescent="0.25">
       <c r="AF6" s="5" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="AG6" s="5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:45" ht="45" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:45" ht="30" x14ac:dyDescent="0.25">
       <c r="AF7" s="5" t="s">
-        <v>124</v>
+        <v>75</v>
       </c>
       <c r="AG7" s="5" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:45" ht="45" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:45" ht="30" x14ac:dyDescent="0.25">
       <c r="AF8" s="5" t="s">
-        <v>77</v>
+        <v>117</v>
       </c>
       <c r="AG8" s="5" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:45" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:45" x14ac:dyDescent="0.25">
       <c r="AF9" s="5" t="s">
-        <v>88</v>
+        <v>119</v>
       </c>
       <c r="AG9" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:45" ht="60" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="10" spans="1:45" x14ac:dyDescent="0.25">
       <c r="AF10" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="AG10" s="5" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:45" ht="30" x14ac:dyDescent="0.25">
       <c r="AF11" s="5" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AG11" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="12" spans="1:45" ht="60" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:45" x14ac:dyDescent="0.25">
       <c r="AF12" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="AG12" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="13" spans="1:45" ht="30" x14ac:dyDescent="0.25">
-      <c r="AF13" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="AG13" s="5" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:45" ht="30" x14ac:dyDescent="0.25">
-      <c r="AF14" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="AG14" s="5" t="s">
-        <v>70</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="AG12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:45" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="AN13" s="5"/>
+      <c r="AO13" s="5"/>
+      <c r="AP13" s="5"/>
+      <c r="AQ13" s="5"/>
+      <c r="AR13" s="5"/>
+      <c r="AS13" s="5"/>
+    </row>
+    <row r="14" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AN14" s="5"/>
+      <c r="AO14" s="5"/>
+      <c r="AP14" s="5"/>
+      <c r="AQ14" s="5"/>
+      <c r="AR14" s="5"/>
+      <c r="AS14" s="5"/>
     </row>
     <row r="15" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="AF15" s="5"/>
-    </row>
-    <row r="16" spans="1:45" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="J16" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="K16" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="M16" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="N16" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="O16" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="P16" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q16" s="5">
-        <v>1</v>
-      </c>
-      <c r="R16" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="S16" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="T16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="U16" s="7">
-        <v>46066</v>
-      </c>
-      <c r="V16" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="W16" s="7">
-        <v>46066</v>
-      </c>
-      <c r="X16" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y16" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z16" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="AA16" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="AB16" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="AC16" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="AD16" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="AE16" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="AF16" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="AG16" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="AH16" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="AI16" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="AJ16" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="AK16" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="AL16" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="AM16" s="5" t="s">
-        <v>41</v>
-      </c>
+      <c r="AN15" s="5"/>
+      <c r="AO15" s="5"/>
+      <c r="AP15" s="5"/>
+      <c r="AQ15" s="5"/>
+      <c r="AR15" s="5"/>
+      <c r="AS15" s="5"/>
+    </row>
+    <row r="16" spans="1:45" x14ac:dyDescent="0.25">
       <c r="AN16" s="5"/>
       <c r="AO16" s="5"/>
       <c r="AP16" s="5"/>
@@ -1268,50 +1145,7 @@
       <c r="AR16" s="5"/>
       <c r="AS16" s="5"/>
     </row>
-    <row r="17" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-      <c r="E17" s="5"/>
-      <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-      <c r="Q17" s="5"/>
-      <c r="R17" s="5"/>
-      <c r="S17" s="5"/>
-      <c r="T17" s="5"/>
-      <c r="U17" s="5"/>
-      <c r="V17" s="5"/>
-      <c r="W17" s="5"/>
-      <c r="X17" s="5"/>
-      <c r="Y17" s="5"/>
-      <c r="Z17" s="5"/>
-      <c r="AA17" s="5"/>
-      <c r="AB17" s="5"/>
-      <c r="AC17" s="5"/>
-      <c r="AD17" s="5"/>
-      <c r="AE17" s="5"/>
-      <c r="AF17" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="AG17" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="AH17" s="5"/>
-      <c r="AI17" s="5"/>
-      <c r="AJ17" s="5"/>
-      <c r="AK17" s="5"/>
-      <c r="AL17" s="5"/>
-      <c r="AM17" s="5"/>
+    <row r="17" spans="40:45" x14ac:dyDescent="0.25">
       <c r="AN17" s="5"/>
       <c r="AO17" s="5"/>
       <c r="AP17" s="5"/>
@@ -1319,50 +1153,7 @@
       <c r="AR17" s="5"/>
       <c r="AS17" s="5"/>
     </row>
-    <row r="18" spans="1:45" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-      <c r="I18" s="5"/>
-      <c r="J18" s="5"/>
-      <c r="K18" s="5"/>
-      <c r="L18" s="5"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
-      <c r="P18" s="5"/>
-      <c r="Q18" s="5"/>
-      <c r="R18" s="5"/>
-      <c r="S18" s="5"/>
-      <c r="T18" s="5"/>
-      <c r="U18" s="5"/>
-      <c r="V18" s="5"/>
-      <c r="W18" s="5"/>
-      <c r="X18" s="5"/>
-      <c r="Y18" s="5"/>
-      <c r="Z18" s="5"/>
-      <c r="AA18" s="5"/>
-      <c r="AB18" s="5"/>
-      <c r="AC18" s="5"/>
-      <c r="AD18" s="5"/>
-      <c r="AE18" s="5"/>
-      <c r="AF18" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="AG18" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="AH18" s="5"/>
-      <c r="AI18" s="5"/>
-      <c r="AJ18" s="5"/>
-      <c r="AK18" s="5"/>
-      <c r="AL18" s="5"/>
-      <c r="AM18" s="5"/>
+    <row r="18" spans="40:45" x14ac:dyDescent="0.25">
       <c r="AN18" s="5"/>
       <c r="AO18" s="5"/>
       <c r="AP18" s="5"/>
@@ -1370,50 +1161,7 @@
       <c r="AR18" s="5"/>
       <c r="AS18" s="5"/>
     </row>
-    <row r="19" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A19" s="5"/>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5"/>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
-      <c r="U19" s="5"/>
-      <c r="V19" s="5"/>
-      <c r="W19" s="5"/>
-      <c r="X19" s="5"/>
-      <c r="Y19" s="5"/>
-      <c r="Z19" s="5"/>
-      <c r="AA19" s="5"/>
-      <c r="AB19" s="5"/>
-      <c r="AC19" s="5"/>
-      <c r="AD19" s="5"/>
-      <c r="AE19" s="5"/>
-      <c r="AF19" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="AG19" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="AH19" s="5"/>
-      <c r="AI19" s="5"/>
-      <c r="AJ19" s="5"/>
-      <c r="AK19" s="5"/>
-      <c r="AL19" s="5"/>
-      <c r="AM19" s="5"/>
+    <row r="19" spans="40:45" x14ac:dyDescent="0.25">
       <c r="AN19" s="5"/>
       <c r="AO19" s="5"/>
       <c r="AP19" s="5"/>
@@ -1421,50 +1169,7 @@
       <c r="AR19" s="5"/>
       <c r="AS19" s="5"/>
     </row>
-    <row r="20" spans="1:45" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-      <c r="R20" s="5"/>
-      <c r="S20" s="5"/>
-      <c r="T20" s="5"/>
-      <c r="U20" s="5"/>
-      <c r="V20" s="5"/>
-      <c r="W20" s="5"/>
-      <c r="X20" s="5"/>
-      <c r="Y20" s="5"/>
-      <c r="Z20" s="5"/>
-      <c r="AA20" s="5"/>
-      <c r="AB20" s="5"/>
-      <c r="AC20" s="5"/>
-      <c r="AD20" s="5"/>
-      <c r="AE20" s="5"/>
-      <c r="AF20" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="AG20" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="AH20" s="5"/>
-      <c r="AI20" s="5"/>
-      <c r="AJ20" s="5"/>
-      <c r="AK20" s="5"/>
-      <c r="AL20" s="5"/>
-      <c r="AM20" s="5"/>
+    <row r="20" spans="40:45" x14ac:dyDescent="0.25">
       <c r="AN20" s="5"/>
       <c r="AO20" s="5"/>
       <c r="AP20" s="5"/>
@@ -1472,50 +1177,7 @@
       <c r="AR20" s="5"/>
       <c r="AS20" s="5"/>
     </row>
-    <row r="21" spans="1:45" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-      <c r="E21" s="5"/>
-      <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-      <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
-      <c r="K21" s="5"/>
-      <c r="L21" s="5"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
-      <c r="P21" s="5"/>
-      <c r="Q21" s="5"/>
-      <c r="R21" s="5"/>
-      <c r="S21" s="5"/>
-      <c r="T21" s="5"/>
-      <c r="U21" s="5"/>
-      <c r="V21" s="5"/>
-      <c r="W21" s="5"/>
-      <c r="X21" s="5"/>
-      <c r="Y21" s="5"/>
-      <c r="Z21" s="5"/>
-      <c r="AA21" s="5"/>
-      <c r="AB21" s="5"/>
-      <c r="AC21" s="5"/>
-      <c r="AD21" s="5"/>
-      <c r="AE21" s="5"/>
-      <c r="AF21" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="AG21" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="AH21" s="5"/>
-      <c r="AI21" s="5"/>
-      <c r="AJ21" s="5"/>
-      <c r="AK21" s="5"/>
-      <c r="AL21" s="5"/>
-      <c r="AM21" s="5"/>
+    <row r="21" spans="40:45" x14ac:dyDescent="0.25">
       <c r="AN21" s="5"/>
       <c r="AO21" s="5"/>
       <c r="AP21" s="5"/>
@@ -1523,162 +1185,503 @@
       <c r="AR21" s="5"/>
       <c r="AS21" s="5"/>
     </row>
-    <row r="22" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-      <c r="Q22" s="5"/>
-      <c r="R22" s="5"/>
-      <c r="S22" s="5"/>
-      <c r="T22" s="5"/>
-      <c r="U22" s="5"/>
-      <c r="V22" s="5"/>
-      <c r="W22" s="5"/>
-      <c r="X22" s="5"/>
-      <c r="Y22" s="5"/>
-      <c r="Z22" s="5"/>
-      <c r="AA22" s="5"/>
-      <c r="AB22" s="5"/>
-      <c r="AC22" s="5"/>
-      <c r="AD22" s="5"/>
-      <c r="AE22" s="5"/>
-      <c r="AF22" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="AG22" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="AH22" s="5"/>
-      <c r="AI22" s="5"/>
-      <c r="AJ22" s="5"/>
-      <c r="AK22" s="5"/>
-      <c r="AL22" s="5"/>
-      <c r="AM22" s="5"/>
-      <c r="AN22" s="5"/>
-      <c r="AO22" s="5"/>
-      <c r="AP22" s="5"/>
-      <c r="AQ22" s="5"/>
-      <c r="AR22" s="5"/>
-      <c r="AS22" s="5"/>
-    </row>
-    <row r="23" spans="1:45" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-      <c r="U23" s="5"/>
-      <c r="V23" s="5"/>
-      <c r="W23" s="5"/>
-      <c r="X23" s="5"/>
-      <c r="Y23" s="5"/>
-      <c r="Z23" s="5"/>
-      <c r="AA23" s="5"/>
-      <c r="AB23" s="5"/>
-      <c r="AC23" s="5"/>
-      <c r="AD23" s="5"/>
-      <c r="AE23" s="5"/>
-      <c r="AF23" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="AG23" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="AH23" s="5"/>
-      <c r="AI23" s="5"/>
-      <c r="AJ23" s="5"/>
-      <c r="AK23" s="5"/>
-      <c r="AL23" s="5"/>
-      <c r="AM23" s="5"/>
-      <c r="AN23" s="5"/>
-      <c r="AO23" s="5"/>
-      <c r="AP23" s="5"/>
-      <c r="AQ23" s="5"/>
-      <c r="AR23" s="5"/>
-      <c r="AS23" s="5"/>
-    </row>
-    <row r="24" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="A24" s="5"/>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="5"/>
-      <c r="R24" s="5"/>
-      <c r="S24" s="5"/>
-      <c r="T24" s="5"/>
-      <c r="U24" s="5"/>
-      <c r="V24" s="5"/>
-      <c r="W24" s="5"/>
-      <c r="X24" s="5"/>
-      <c r="Y24" s="5"/>
-      <c r="Z24" s="5"/>
-      <c r="AA24" s="5"/>
-      <c r="AB24" s="5"/>
-      <c r="AC24" s="5"/>
-      <c r="AD24" s="5"/>
-      <c r="AE24" s="5"/>
-      <c r="AF24" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="AG24" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="AH24" s="5"/>
-      <c r="AI24" s="5"/>
-      <c r="AJ24" s="5"/>
-      <c r="AK24" s="5"/>
-      <c r="AL24" s="5"/>
-      <c r="AM24" s="5"/>
-      <c r="AN24" s="5"/>
-      <c r="AO24" s="5"/>
-      <c r="AP24" s="5"/>
-      <c r="AQ24" s="5"/>
-      <c r="AR24" s="5"/>
-      <c r="AS24" s="5"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57D70074-4EA7-45FE-BFA1-9D9428617F8C}">
+  <dimension ref="A2:AM11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="2" spans="1:39" ht="360" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q2" s="5">
+        <v>1</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="S2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="T2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="U2" s="7">
+        <v>46066</v>
+      </c>
+      <c r="V2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" s="7">
+        <v>46066</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="Y2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z2" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="AA2" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="AC2" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="AD2" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="AE2" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="AF2" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="AG2" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="AH2" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AI2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AJ2" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="AK2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="AL2" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="AM2" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:39" ht="120" x14ac:dyDescent="0.25">
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
+      <c r="P3" s="5"/>
+      <c r="Q3" s="5"/>
+      <c r="R3" s="5"/>
+      <c r="S3" s="5"/>
+      <c r="T3" s="5"/>
+      <c r="U3" s="5"/>
+      <c r="V3" s="5"/>
+      <c r="W3" s="5"/>
+      <c r="X3" s="5"/>
+      <c r="Y3" s="5"/>
+      <c r="Z3" s="5"/>
+      <c r="AA3" s="5"/>
+      <c r="AB3" s="5"/>
+      <c r="AC3" s="5"/>
+      <c r="AD3" s="5"/>
+      <c r="AE3" s="5"/>
+      <c r="AF3" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="AG3" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="AH3" s="5"/>
+      <c r="AI3" s="5"/>
+      <c r="AJ3" s="5"/>
+      <c r="AK3" s="5"/>
+      <c r="AL3" s="5"/>
+      <c r="AM3" s="5"/>
+    </row>
+    <row r="4" spans="1:39" ht="240" x14ac:dyDescent="0.25">
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
+      <c r="P4" s="5"/>
+      <c r="Q4" s="5"/>
+      <c r="R4" s="5"/>
+      <c r="S4" s="5"/>
+      <c r="T4" s="5"/>
+      <c r="U4" s="5"/>
+      <c r="V4" s="5"/>
+      <c r="W4" s="5"/>
+      <c r="X4" s="5"/>
+      <c r="Y4" s="5"/>
+      <c r="Z4" s="5"/>
+      <c r="AA4" s="5"/>
+      <c r="AB4" s="5"/>
+      <c r="AC4" s="5"/>
+      <c r="AD4" s="5"/>
+      <c r="AE4" s="5"/>
+      <c r="AF4" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="AG4" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="AH4" s="5"/>
+      <c r="AI4" s="5"/>
+      <c r="AJ4" s="5"/>
+      <c r="AK4" s="5"/>
+      <c r="AL4" s="5"/>
+      <c r="AM4" s="5"/>
+    </row>
+    <row r="5" spans="1:39" ht="120" x14ac:dyDescent="0.25">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
+      <c r="P5" s="5"/>
+      <c r="Q5" s="5"/>
+      <c r="R5" s="5"/>
+      <c r="S5" s="5"/>
+      <c r="T5" s="5"/>
+      <c r="U5" s="5"/>
+      <c r="V5" s="5"/>
+      <c r="W5" s="5"/>
+      <c r="X5" s="5"/>
+      <c r="Y5" s="5"/>
+      <c r="Z5" s="5"/>
+      <c r="AA5" s="5"/>
+      <c r="AB5" s="5"/>
+      <c r="AC5" s="5"/>
+      <c r="AD5" s="5"/>
+      <c r="AE5" s="5"/>
+      <c r="AF5" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="AG5" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="AH5" s="5"/>
+      <c r="AI5" s="5"/>
+      <c r="AJ5" s="5"/>
+      <c r="AK5" s="5"/>
+      <c r="AL5" s="5"/>
+      <c r="AM5" s="5"/>
+    </row>
+    <row r="6" spans="1:39" ht="150" x14ac:dyDescent="0.25">
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5"/>
+      <c r="W6" s="5"/>
+      <c r="X6" s="5"/>
+      <c r="Y6" s="5"/>
+      <c r="Z6" s="5"/>
+      <c r="AA6" s="5"/>
+      <c r="AB6" s="5"/>
+      <c r="AC6" s="5"/>
+      <c r="AD6" s="5"/>
+      <c r="AE6" s="5"/>
+      <c r="AF6" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="AG6" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="AH6" s="5"/>
+      <c r="AI6" s="5"/>
+      <c r="AJ6" s="5"/>
+      <c r="AK6" s="5"/>
+      <c r="AL6" s="5"/>
+      <c r="AM6" s="5"/>
+    </row>
+    <row r="7" spans="1:39" ht="165" x14ac:dyDescent="0.25">
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5"/>
+      <c r="T7" s="5"/>
+      <c r="U7" s="5"/>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="5"/>
+      <c r="Y7" s="5"/>
+      <c r="Z7" s="5"/>
+      <c r="AA7" s="5"/>
+      <c r="AB7" s="5"/>
+      <c r="AC7" s="5"/>
+      <c r="AD7" s="5"/>
+      <c r="AE7" s="5"/>
+      <c r="AF7" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="AG7" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="AH7" s="5"/>
+      <c r="AI7" s="5"/>
+      <c r="AJ7" s="5"/>
+      <c r="AK7" s="5"/>
+      <c r="AL7" s="5"/>
+      <c r="AM7" s="5"/>
+    </row>
+    <row r="8" spans="1:39" ht="120" x14ac:dyDescent="0.25">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5"/>
+      <c r="W8" s="5"/>
+      <c r="X8" s="5"/>
+      <c r="Y8" s="5"/>
+      <c r="Z8" s="5"/>
+      <c r="AA8" s="5"/>
+      <c r="AB8" s="5"/>
+      <c r="AC8" s="5"/>
+      <c r="AD8" s="5"/>
+      <c r="AE8" s="5"/>
+      <c r="AF8" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="AG8" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="AH8" s="5"/>
+      <c r="AI8" s="5"/>
+      <c r="AJ8" s="5"/>
+      <c r="AK8" s="5"/>
+      <c r="AL8" s="5"/>
+      <c r="AM8" s="5"/>
+    </row>
+    <row r="9" spans="1:39" ht="255" x14ac:dyDescent="0.25">
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
+      <c r="P9" s="5"/>
+      <c r="Q9" s="5"/>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
+      <c r="V9" s="5"/>
+      <c r="W9" s="5"/>
+      <c r="X9" s="5"/>
+      <c r="Y9" s="5"/>
+      <c r="Z9" s="5"/>
+      <c r="AA9" s="5"/>
+      <c r="AB9" s="5"/>
+      <c r="AC9" s="5"/>
+      <c r="AD9" s="5"/>
+      <c r="AE9" s="5"/>
+      <c r="AF9" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="AG9" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="AH9" s="5"/>
+      <c r="AI9" s="5"/>
+      <c r="AJ9" s="5"/>
+      <c r="AK9" s="5"/>
+      <c r="AL9" s="5"/>
+      <c r="AM9" s="5"/>
+    </row>
+    <row r="10" spans="1:39" ht="105" x14ac:dyDescent="0.25">
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="5"/>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
+      <c r="V10" s="5"/>
+      <c r="W10" s="5"/>
+      <c r="X10" s="5"/>
+      <c r="Y10" s="5"/>
+      <c r="Z10" s="5"/>
+      <c r="AA10" s="5"/>
+      <c r="AB10" s="5"/>
+      <c r="AC10" s="5"/>
+      <c r="AD10" s="5"/>
+      <c r="AE10" s="5"/>
+      <c r="AF10" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG10" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="AH10" s="5"/>
+      <c r="AI10" s="5"/>
+      <c r="AJ10" s="5"/>
+      <c r="AK10" s="5"/>
+      <c r="AL10" s="5"/>
+      <c r="AM10" s="5"/>
+    </row>
+    <row r="11" spans="1:39" x14ac:dyDescent="0.25">
+      <c r="Q11" s="1"/>
+      <c r="U11" s="2"/>
+      <c r="W11" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="AF16" r:id="rId1" tooltip="https://www.cse.lk/" display="https://www.cse.lk/" xr:uid="{7313FD41-28FB-4762-9CAE-2056423D089D}"/>
+    <hyperlink ref="AF2" r:id="rId1" tooltip="https://www.cse.lk/" display="https://www.cse.lk/" xr:uid="{7313FD41-28FB-4762-9CAE-2056423D089D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>